<commit_message>
Check_Registered - Version 1.0.1
</commit_message>
<xml_diff>
--- a/Check_Registered/Data/Documents/Config.xlsx
+++ b/Check_Registered/Data/Documents/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UiPathProjects\UiPathAutomation\Check_Registered\Data\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UiPath_GitProjects\IGR_Project\IGR_Master\Data\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69095C8-3EEE-4317-9CDC-5CBFA0623562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69576EC-AF35-46A1-BF4D-DFA995D05695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="119">
   <si>
     <t>Name</t>
   </si>
@@ -354,7 +354,31 @@
     <t>Description (Assets will always overwrite other config)</t>
   </si>
   <si>
-    <t>D:\UiPathProjects\UiPathAutomation\Check_Registered\Data\Documents</t>
+    <t>AdPDetailsSheet</t>
+  </si>
+  <si>
+    <t>AdPDetails</t>
+  </si>
+  <si>
+    <t>C:\Users\DeokateLaxman\Documents\UiPathAutomation\IGR_Master\Data\Documents</t>
+  </si>
+  <si>
+    <t>ServiceProvider</t>
+  </si>
+  <si>
+    <t>Prof. Laxman Jagannath Deokate</t>
+  </si>
+  <si>
+    <t>WebMessage</t>
+  </si>
+  <si>
+    <t>Please share your valuable review/feedback and 5 star rating on below link which Will help us to improve our services</t>
+  </si>
+  <si>
+    <t>WebLink</t>
+  </si>
+  <si>
+    <t>https://g.page/online-registered-rent-agree-117?share</t>
   </si>
 </sst>
 </file>
@@ -703,13 +727,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z993"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:Z998"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
-    <col min="2" max="2" width="95.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="43.54296875" customWidth="1"/>
+    <col min="2" max="2" width="95.1796875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="81.453125" customWidth="1"/>
+    <col min="4" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -746,7 +770,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" s="4" customFormat="1" ht="15.75">
+    <row r="2" spans="1:26" s="4" customFormat="1" ht="15.5">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -754,7 +778,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="18.75">
+    <row r="3" spans="1:26" ht="18.5">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -791,7 +815,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
@@ -903,189 +927,217 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="20" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A20" t="s">
-        <v>35</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
+    <row r="19" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B19" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>41</v>
-      </c>
-      <c r="B23" t="s">
-        <v>42</v>
+        <v>39</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>43</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
+      </c>
+      <c r="B24" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1">
       <c r="A25" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A26" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B26" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="27" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="28" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A28" t="s">
-        <v>47</v>
-      </c>
-      <c r="B28" s="2">
-        <v>9011092282</v>
-      </c>
-    </row>
+    <row r="28" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>48</v>
+        <v>113</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A30" t="s">
+        <v>115</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
     <row r="31" spans="1:2" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>50</v>
+        <v>117</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>51</v>
+        <v>118</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>52</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="34" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A34" t="s">
-        <v>54</v>
-      </c>
-      <c r="B34" s="2">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A35" t="s">
-        <v>55</v>
-      </c>
-      <c r="B35" s="2">
-        <v>300</v>
-      </c>
-    </row>
+        <v>47</v>
+      </c>
+      <c r="B32" s="2">
+        <v>9011092282</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A33" t="s">
+        <v>48</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="35" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="36" spans="1:3" ht="14.25" customHeight="1">
       <c r="A36" t="s">
-        <v>56</v>
-      </c>
-      <c r="B36" t="s">
-        <v>57</v>
+        <v>50</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="14.25" customHeight="1">
       <c r="A37" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="39" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="39" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A39" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="2">
+        <v>1000</v>
+      </c>
+    </row>
     <row r="40" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B40" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="14.25" customHeight="1"/>
+      <c r="A40" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" s="2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A41" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" t="s">
+        <v>57</v>
+      </c>
+    </row>
     <row r="42" spans="1:3" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>61</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C42" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A43" t="s">
-        <v>64</v>
-      </c>
-      <c r="B43" s="7"/>
-      <c r="C43" t="s">
-        <v>65</v>
-      </c>
-    </row>
+        <v>58</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="44" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="45" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A45" t="s">
+      <c r="B45" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="47" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A47" t="s">
+        <v>61</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C47" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A48" t="s">
+        <v>64</v>
+      </c>
+      <c r="B48" s="7"/>
+      <c r="C48" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="50" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A50" t="s">
         <v>66</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B50" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C50" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A46" t="s">
+    <row r="51" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A51" t="s">
         <v>69</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B51" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="48" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1"/>
-    <row r="63" ht="14.25" customHeight="1"/>
-    <row r="64" ht="14.25" customHeight="1"/>
+    <row r="52" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="53" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="54" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="55" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="56" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="57" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="58" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="59" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="60" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="61" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="62" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="63" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="64" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="65" ht="14.25" customHeight="1"/>
     <row r="66" ht="14.25" customHeight="1"/>
     <row r="67" ht="14.25" customHeight="1"/>
@@ -2015,6 +2067,11 @@
     <row r="991" ht="14.25" customHeight="1"/>
     <row r="992" ht="14.25" customHeight="1"/>
     <row r="993" ht="14.25" customHeight="1"/>
+    <row r="994" ht="14.25" customHeight="1"/>
+    <row r="995" ht="14.25" customHeight="1"/>
+    <row r="996" ht="14.25" customHeight="1"/>
+    <row r="997" ht="14.25" customHeight="1"/>
+    <row r="998" ht="14.25" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -2024,12 +2081,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="75.453125" customWidth="1"/>
+    <col min="4" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -2066,7 +2123,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="29">
       <c r="A2" t="s">
         <v>71</v>
       </c>
@@ -2077,7 +2134,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.5">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -2191,7 +2248,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="45">
+    <row r="17" spans="1:3" ht="29">
       <c r="A17" t="s">
         <v>100</v>
       </c>
@@ -3216,12 +3273,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" customWidth="1"/>
-    <col min="4" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="31.81640625" customWidth="1"/>
+    <col min="2" max="2" width="30.1796875" customWidth="1"/>
+    <col min="3" max="3" width="60.26953125" customWidth="1"/>
+    <col min="4" max="26" width="65.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">

</xml_diff>